<commit_message>
feat(excel): support parallel links and degree associations
Allow Excel topology files to define multiple bidirectional links between
the same pair of nodes.

Assign pair identifiers to parallel links, equipment and ROADM degrees
according to their source row order. Propagate these identifiers to generated
JSON UIDs and preserve the association between parallel ROADM degrees.

Duplicate ILA and FUSED nodes when they are traversed by different link pairs
and validate inconsistent parallel-link, equipment and ROADM definitions.

Also preserve ROADM degree associations when redesigning a filtered topology.

Add tests covering valid and invalid parallel link configurations.

Signed-off-by: EstherLerouzic <esther.lerouzic@orange.com>
Change-Id: I3c99765d378f72f5c36173de9577ba4690eb0f21
</commit_message>
<xml_diff>
--- a/tests/data/wrong_topo_duplicate_eqpt.xlsx
+++ b/tests/data/wrong_topo_duplicate_eqpt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\partage_vm\jeuTestWebapi\request-run\wrong_xls\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\user\workspace\TIP\test\oopt-gnpy\tests\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B8D59A-E4EA-4E13-9E89-6993610291AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65FC688B-C9D9-4F8A-8931-E212DE0BBF37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="20376" windowHeight="12096" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>

</xml_diff>